<commit_message>
add synthesis tab and download button
</commit_message>
<xml_diff>
--- a/asset/tableau de synthese.xlsx
+++ b/asset/tableau de synthese.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="42">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -52,27 +52,7 @@
     <t xml:space="preserve">☑ SLAM</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="18"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Adresse URL du portfolio : </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="18"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://mehdimaallou.me</t>
-    </r>
+    <t xml:space="preserve">Adresse URL du portfolio : https://mehdimaallou.me</t>
   </si>
   <si>
     <t xml:space="preserve">Compétences mises en œuvre
@@ -167,7 +147,30 @@
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
+    <t xml:space="preserve">Réalisation d’un site web et d’une base de données administrant les données d’un projet de robot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Du 15/05/23
+Au 16/06/23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réalisation d’une interface utilisateur en Réalité Virtuelle sur une page web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmation d’un Raspberry PI-0 permettant la saisi automatique de mot de passe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de seconde année</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réalisation d’un site web et d’une base de données administrant les données des visiteurs de la MJC de bolbec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Du 08/01/2024
+Au 26/02/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installation et administration d’un serveur web dédié</t>
   </si>
 </sst>
 </file>
@@ -259,7 +262,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="15"/>
+      <sz val="16"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -596,156 +599,148 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1008,483 +1003,553 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="18.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="9" style="0" width="10.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="9" style="2" width="10.91"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="44" style="1" width="10.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="2"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="6" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" s="16" customFormat="true" ht="324.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="14" t="s">
+    <row r="7" s="17" customFormat="true" ht="324.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="16" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" s="16" customFormat="true" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+    <row r="8" s="17" customFormat="true" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-    </row>
-    <row r="9" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+    </row>
+    <row r="9" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="21"/>
-    </row>
-    <row r="10" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="C9" s="21"/>
+      <c r="D9" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="21"/>
+      <c r="H9" s="22"/>
+    </row>
+    <row r="10" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="20"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="21"/>
+      <c r="H10" s="22"/>
+    </row>
+    <row r="11" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="21"/>
-    </row>
-    <row r="12" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="C11" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="22"/>
+    </row>
+    <row r="12" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="25"/>
-    </row>
-    <row r="14" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="25"/>
-    </row>
-    <row r="15" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="25"/>
-    </row>
-    <row r="16" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="25"/>
-    </row>
-    <row r="17" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="25"/>
-    </row>
-    <row r="18" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="25"/>
-    </row>
-    <row r="19" s="16" customFormat="true" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="26" t="s">
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="21"/>
+      <c r="H12" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="26"/>
+    </row>
+    <row r="14" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="26"/>
+    </row>
+    <row r="15" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="26"/>
+    </row>
+    <row r="16" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="26"/>
+    </row>
+    <row r="17" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="26"/>
+    </row>
+    <row r="18" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="26"/>
+    </row>
+    <row r="19" s="17" customFormat="true" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-    </row>
-    <row r="20" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="25"/>
-    </row>
-    <row r="21" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="25"/>
-    </row>
-    <row r="22" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="25"/>
-    </row>
-    <row r="23" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="25"/>
-    </row>
-    <row r="24" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="25"/>
-    </row>
-    <row r="25" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="25"/>
-    </row>
-    <row r="26" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="25"/>
-    </row>
-    <row r="27" s="16" customFormat="true" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="s">
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+    </row>
+    <row r="20" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-    </row>
-    <row r="28" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="25"/>
-    </row>
-    <row r="29" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="25"/>
-    </row>
-    <row r="30" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="25"/>
-    </row>
-    <row r="31" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="25"/>
-    </row>
-    <row r="32" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="25"/>
-    </row>
-    <row r="33" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="30"/>
-    </row>
-    <row r="34" s="16" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="B20" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="26"/>
+    </row>
+    <row r="21" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" s="26"/>
+    </row>
+    <row r="22" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="26"/>
+    </row>
+    <row r="23" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="26"/>
+    </row>
+    <row r="24" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="26"/>
+    </row>
+    <row r="25" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="26"/>
+    </row>
+    <row r="26" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="26"/>
+    </row>
+    <row r="27" s="17" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+    </row>
+    <row r="28" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G29" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="26"/>
+    </row>
+    <row r="31" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="26"/>
+    </row>
+    <row r="32" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="26"/>
+    </row>
+    <row r="33" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="26"/>
+    </row>
+    <row r="34" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="29"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="32"/>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="35"/>
-      <c r="B35" s="36"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="16"/>
-      <c r="Q35" s="16"/>
-      <c r="R35" s="16"/>
-      <c r="S35" s="16"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
-      <c r="V35" s="16"/>
-      <c r="W35" s="16"/>
-      <c r="X35" s="16"/>
-      <c r="Y35" s="16"/>
-      <c r="Z35" s="16"/>
-      <c r="AA35" s="16"/>
-      <c r="AB35" s="16"/>
-      <c r="AC35" s="16"/>
-      <c r="AD35" s="16"/>
-      <c r="AE35" s="16"/>
-      <c r="AF35" s="16"/>
-      <c r="AG35" s="16"/>
-      <c r="AH35" s="16"/>
-      <c r="AI35" s="16"/>
-      <c r="AJ35" s="16"/>
-      <c r="AK35" s="16"/>
-      <c r="AL35" s="16"/>
-      <c r="AM35" s="16"/>
-      <c r="AN35" s="16"/>
-      <c r="AO35" s="16"/>
-      <c r="AP35" s="16"/>
-      <c r="AQ35" s="16"/>
+      <c r="A35" s="33"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="35"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17"/>
+      <c r="P35" s="17"/>
+      <c r="Q35" s="17"/>
+      <c r="R35" s="17"/>
+      <c r="S35" s="17"/>
+      <c r="T35" s="17"/>
+      <c r="U35" s="17"/>
+      <c r="V35" s="17"/>
+      <c r="W35" s="17"/>
+      <c r="X35" s="17"/>
+      <c r="Y35" s="17"/>
+      <c r="Z35" s="17"/>
+      <c r="AA35" s="17"/>
+      <c r="AB35" s="17"/>
+      <c r="AC35" s="17"/>
+      <c r="AD35" s="17"/>
+      <c r="AE35" s="17"/>
+      <c r="AF35" s="17"/>
+      <c r="AG35" s="17"/>
+      <c r="AH35" s="17"/>
+      <c r="AI35" s="17"/>
+      <c r="AJ35" s="17"/>
+      <c r="AK35" s="17"/>
+      <c r="AL35" s="17"/>
+      <c r="AM35" s="17"/>
+      <c r="AN35" s="17"/>
+      <c r="AO35" s="17"/>
+      <c r="AP35" s="17"/>
+      <c r="AQ35" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1502,7 +1567,7 @@
     <mergeCell ref="A27:H27"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1" display="https://mehdimaallou.me"/>
+    <hyperlink ref="A5" r:id="rId1" display="Adresse URL du portfolio : https://mehdimaallou.me"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>